<commit_message>
Fixed max capacity constraint
</commit_message>
<xml_diff>
--- a/data/Ammonia_paper/model_inputs/Data_ammonia_paper.xlsx
+++ b/data/Ammonia_paper/model_inputs/Data_ammonia_paper.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA624466-5CAF-4125-999B-B70E5CDA2366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{DA624466-5CAF-4125-999B-B70E5CDA2366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED6D85D9-FC28-4244-9806-BA15EB30CF2C}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-1620" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_base_case" sheetId="79" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="155">
   <si>
     <t>Red: Don't change the name without changing the Julia code</t>
   </si>
@@ -135,9 +135,6 @@
     <t>Solar tracking</t>
   </si>
   <si>
-    <t>RPU_Solar_track</t>
-  </si>
-  <si>
     <t>RPU_Solar_fixed</t>
   </si>
   <si>
@@ -505,6 +502,9 @@
   </si>
   <si>
     <t>Yearly demand (output)</t>
+  </si>
+  <si>
+    <t>RPU_Solar_tracking</t>
   </si>
 </sst>
 </file>
@@ -989,7 +989,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+    <cellStyle name="Per cent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -1033,6 +1033,9 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Sources"/>
       <sheetName val="Fuel production cost"/>
@@ -1103,6 +1106,10 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1380,7 +1387,7 @@
     <col min="11" max="11" width="9.36328125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.7265625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12" style="2" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="36" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="26.453125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="25.453125" bestFit="1" customWidth="1"/>
@@ -1404,16 +1411,16 @@
       <c r="D1" s="114"/>
       <c r="E1" s="115"/>
       <c r="F1" s="44" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G1" s="44" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H1" s="44" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I1" s="45" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J1" s="100" t="s">
         <v>2</v>
@@ -1427,44 +1434,44 @@
       <c r="M1" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="45" t="s">
+      <c r="N1" s="46" t="s">
         <v>6</v>
       </c>
       <c r="O1" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="P1" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="P1" s="47" t="s">
+      <c r="Q1" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="Q1" s="47" t="s">
+      <c r="R1" s="47" t="s">
         <v>45</v>
       </c>
-      <c r="R1" s="47" t="s">
+      <c r="S1" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="S1" s="47" t="s">
+      <c r="T1" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="T1" s="47" t="s">
+      <c r="U1" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="V1" s="47" t="s">
+        <v>97</v>
+      </c>
+      <c r="W1" s="47" t="s">
+        <v>136</v>
+      </c>
+      <c r="X1" s="47" t="s">
+        <v>98</v>
+      </c>
+      <c r="Y1" s="47" t="s">
+        <v>99</v>
+      </c>
+      <c r="Z1" s="46" t="s">
         <v>48</v>
-      </c>
-      <c r="U1" s="47" t="s">
-        <v>97</v>
-      </c>
-      <c r="V1" s="47" t="s">
-        <v>98</v>
-      </c>
-      <c r="W1" s="47" t="s">
-        <v>137</v>
-      </c>
-      <c r="X1" s="47" t="s">
-        <v>99</v>
-      </c>
-      <c r="Y1" s="47" t="s">
-        <v>100</v>
-      </c>
-      <c r="Z1" s="46" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:26" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1572,34 +1579,34 @@
       <c r="C3" s="118"/>
       <c r="D3" s="117"/>
       <c r="E3" s="34" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J3" s="101" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="M3" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N3" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O3" s="3">
         <v>2020</v>
@@ -1705,7 +1712,7 @@
         <v>Electrical consumption (kWh/output)2020</v>
       </c>
       <c r="U4" s="15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="V4" s="15" t="str">
         <f t="shared" ref="V4:Z4" si="3">V2&amp;V3</f>
@@ -1824,13 +1831,13 @@
         <v>11</v>
       </c>
       <c r="B6" s="57" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C6" s="58" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D6" s="59" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E6" s="9">
         <f t="shared" ref="E6:E36" si="7">ROW(D6)-ROW($E$5)</f>
@@ -1840,10 +1847,10 @@
         <v>1</v>
       </c>
       <c r="G6" s="60" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H6" s="60" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I6" s="62">
         <f>430*10^6</f>
@@ -1862,8 +1869,8 @@
       <c r="M6" s="62">
         <v>0</v>
       </c>
-      <c r="N6" s="62">
-        <v>20000</v>
+      <c r="N6" s="60" t="s">
+        <v>67</v>
       </c>
       <c r="O6" s="98">
         <v>5.2910052910052912</v>
@@ -1905,13 +1912,13 @@
     <row r="7" spans="1:26" s="62" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="116"/>
       <c r="B7" s="57" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C7" s="58" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D7" s="59" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E7" s="9">
         <f>ROW(D7)-ROW($E$5)</f>
@@ -1921,10 +1928,10 @@
         <v>1</v>
       </c>
       <c r="G7" s="60" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H7" s="60" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I7" s="62">
         <f>430*10^6</f>
@@ -1943,9 +1950,9 @@
       <c r="M7" s="62">
         <v>0</v>
       </c>
-      <c r="N7" s="62">
+      <c r="N7" s="60" t="str">
         <f>N6</f>
-        <v>20000</v>
+        <v>None</v>
       </c>
       <c r="O7" s="98">
         <v>5.2910052910052912</v>
@@ -1987,13 +1994,13 @@
     <row r="8" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A8" s="116"/>
       <c r="B8" s="19" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E8" s="9">
         <f t="shared" si="7"/>
@@ -2003,10 +2010,10 @@
         <v>1</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -2023,8 +2030,8 @@
       <c r="M8">
         <v>0</v>
       </c>
-      <c r="N8">
-        <v>400000</v>
+      <c r="N8" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O8">
         <v>0</v>
@@ -2066,13 +2073,13 @@
     <row r="9" spans="1:26" s="75" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="116"/>
       <c r="B9" s="71" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C9" s="72" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D9" s="73" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E9" s="9">
         <f t="shared" si="7"/>
@@ -2082,10 +2089,10 @@
         <v>1</v>
       </c>
       <c r="G9" s="74" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H9" s="74" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I9" s="75">
         <v>0</v>
@@ -2103,8 +2110,8 @@
       <c r="M9" s="75">
         <v>1</v>
       </c>
-      <c r="N9" s="75">
-        <v>20000</v>
+      <c r="N9" s="74" t="s">
+        <v>67</v>
       </c>
       <c r="O9" s="75">
         <v>6.7000000000000004E-2</v>
@@ -2146,13 +2153,13 @@
     <row r="10" spans="1:26" s="83" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="116"/>
       <c r="B10" s="79" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C10" s="80" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D10" s="81" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E10" s="9">
         <f t="shared" si="7"/>
@@ -2162,10 +2169,10 @@
         <v>1</v>
       </c>
       <c r="G10" s="82" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H10" s="82" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I10" s="83">
         <v>0</v>
@@ -2183,9 +2190,9 @@
       <c r="M10" s="83">
         <v>1</v>
       </c>
-      <c r="N10" s="83">
+      <c r="N10" s="82" t="str">
         <f>N9</f>
-        <v>20000</v>
+        <v>None</v>
       </c>
       <c r="O10" s="83">
         <v>6.7000000000000004E-2</v>
@@ -2227,10 +2234,10 @@
     <row r="11" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A11" s="116"/>
       <c r="B11" s="19" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>21</v>
@@ -2243,10 +2250,10 @@
         <v>1</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I11" s="43">
         <v>0</v>
@@ -2263,9 +2270,9 @@
       <c r="M11">
         <v>-1</v>
       </c>
-      <c r="N11">
+      <c r="N11" s="2" t="str">
         <f>N9</f>
-        <v>20000</v>
+        <v>None</v>
       </c>
       <c r="O11" s="43">
         <v>0</v>
@@ -2307,10 +2314,10 @@
     <row r="12" spans="1:26" s="42" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="116"/>
       <c r="B12" s="64" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C12" s="106" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D12" s="66" t="s">
         <v>24</v>
@@ -2323,10 +2330,10 @@
         <v>1</v>
       </c>
       <c r="G12" s="67" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H12" s="67" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I12" s="42">
         <v>0</v>
@@ -2344,9 +2351,8 @@
       <c r="M12" s="42">
         <v>0</v>
       </c>
-      <c r="N12" s="42">
-        <f>9*N9</f>
-        <v>180000</v>
+      <c r="N12" s="67" t="s">
+        <v>67</v>
       </c>
       <c r="O12" s="42">
         <v>7.76</v>
@@ -2391,7 +2397,7 @@
         <v>18</v>
       </c>
       <c r="C13" s="65" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D13" s="66" t="s">
         <v>22</v>
@@ -2404,10 +2410,10 @@
         <v>1</v>
       </c>
       <c r="G13" s="67" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H13" s="67" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I13" s="88">
         <v>0</v>
@@ -2424,9 +2430,8 @@
       <c r="M13" s="42">
         <v>0</v>
       </c>
-      <c r="N13" s="42">
-        <f>N18</f>
-        <v>2000000</v>
+      <c r="N13" s="67" t="s">
+        <v>67</v>
       </c>
       <c r="O13" s="88">
         <v>0</v>
@@ -2471,7 +2476,7 @@
         <v>19</v>
       </c>
       <c r="C14" s="106" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D14" s="66" t="s">
         <v>23</v>
@@ -2484,10 +2489,10 @@
         <v>1</v>
       </c>
       <c r="G14" s="67" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H14" s="67" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I14" s="88">
         <v>0</v>
@@ -2504,9 +2509,8 @@
       <c r="M14" s="88">
         <v>0</v>
       </c>
-      <c r="N14" s="42">
-        <f>N18</f>
-        <v>2000000</v>
+      <c r="N14" s="67" t="s">
+        <v>67</v>
       </c>
       <c r="O14" s="88">
         <v>0</v>
@@ -2551,10 +2555,10 @@
         <v>13</v>
       </c>
       <c r="C15" s="52" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D15" s="91" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E15" s="9">
         <f t="shared" si="7"/>
@@ -2564,10 +2568,10 @@
         <v>1</v>
       </c>
       <c r="G15" s="53" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H15" s="53" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I15" s="54">
         <v>0</v>
@@ -2584,8 +2588,8 @@
       <c r="M15" s="54">
         <v>-1</v>
       </c>
-      <c r="N15" s="54">
-        <v>20000</v>
+      <c r="N15" s="53" t="s">
+        <v>67</v>
       </c>
       <c r="O15" s="56">
         <v>0</v>
@@ -2630,10 +2634,10 @@
         <v>14</v>
       </c>
       <c r="C16" s="52" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D16" s="91" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E16" s="9">
         <f t="shared" si="7"/>
@@ -2643,10 +2647,10 @@
         <v>1</v>
       </c>
       <c r="G16" s="53" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H16" s="53" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I16" s="54">
         <v>0</v>
@@ -2663,8 +2667,8 @@
       <c r="M16" s="54">
         <v>1</v>
       </c>
-      <c r="N16" s="54">
-        <v>20000</v>
+      <c r="N16" s="53" t="s">
+        <v>67</v>
       </c>
       <c r="O16" s="56">
         <v>0</v>
@@ -2709,10 +2713,10 @@
         <v>15</v>
       </c>
       <c r="C17" s="93" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D17" s="94" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E17" s="90">
         <f t="shared" si="7"/>
@@ -2722,10 +2726,10 @@
         <v>1</v>
       </c>
       <c r="G17" s="95" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H17" s="95" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I17" s="96">
         <v>0</v>
@@ -2742,8 +2746,8 @@
       <c r="M17" s="96">
         <v>0</v>
       </c>
-      <c r="N17" s="96">
-        <v>20000000</v>
+      <c r="N17" s="95" t="s">
+        <v>67</v>
       </c>
       <c r="O17" s="96">
         <v>0</v>
@@ -2787,10 +2791,10 @@
         <v>16</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>29</v>
@@ -2803,10 +2807,10 @@
         <v>1</v>
       </c>
       <c r="G18" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H18" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I18">
         <v>0</v>
@@ -2823,8 +2827,8 @@
       <c r="M18">
         <v>0</v>
       </c>
-      <c r="N18">
-        <v>2000000</v>
+      <c r="N18" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O18" s="10">
         <v>0</v>
@@ -2866,10 +2870,10 @@
     <row r="19" spans="1:26" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="116"/>
       <c r="B19" s="12" t="s">
-        <v>31</v>
+        <v>154</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>30</v>
@@ -2882,10 +2886,10 @@
         <v>1</v>
       </c>
       <c r="G19" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H19" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I19">
         <v>0</v>
@@ -2902,9 +2906,8 @@
       <c r="M19">
         <v>0</v>
       </c>
-      <c r="N19">
-        <f t="shared" ref="N19:N32" si="8">$N$18</f>
-        <v>2000000</v>
+      <c r="N19" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O19" s="10">
         <v>0</v>
@@ -2950,10 +2953,10 @@
         <v>RPU_ON_SP198-HH100</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E20" s="9">
         <f t="shared" si="7"/>
@@ -2963,10 +2966,10 @@
         <v>1</v>
       </c>
       <c r="G20" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H20" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I20">
         <v>0</v>
@@ -2983,9 +2986,8 @@
       <c r="M20">
         <v>0</v>
       </c>
-      <c r="N20">
-        <f t="shared" si="8"/>
-        <v>2000000</v>
+      <c r="N20" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O20" s="10">
         <v>0</v>
@@ -3027,14 +3029,14 @@
     <row r="21" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A21" s="116"/>
       <c r="B21" s="12" t="str">
-        <f t="shared" ref="B21:B31" si="9">CONCATENATE("RPU_"&amp;D21)</f>
+        <f t="shared" ref="B21:B31" si="8">CONCATENATE("RPU_"&amp;D21)</f>
         <v>RPU_ON_SP198-HH150</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E21" s="9">
         <f t="shared" si="7"/>
@@ -3044,10 +3046,10 @@
         <v>1</v>
       </c>
       <c r="G21" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H21" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I21">
         <v>0</v>
@@ -3064,9 +3066,8 @@
       <c r="M21">
         <v>0</v>
       </c>
-      <c r="N21">
-        <f t="shared" si="8"/>
-        <v>2000000</v>
+      <c r="N21" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O21" s="10">
         <v>0</v>
@@ -3108,14 +3109,14 @@
     <row r="22" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A22" s="116"/>
       <c r="B22" s="12" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>RPU_ON_SP237-HH100</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E22" s="9">
         <f t="shared" si="7"/>
@@ -3125,10 +3126,10 @@
         <v>1</v>
       </c>
       <c r="G22" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I22">
         <v>0</v>
@@ -3145,9 +3146,8 @@
       <c r="M22">
         <v>0</v>
       </c>
-      <c r="N22">
-        <f t="shared" si="8"/>
-        <v>2000000</v>
+      <c r="N22" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O22" s="10">
         <v>0</v>
@@ -3189,14 +3189,14 @@
     <row r="23" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A23" s="116"/>
       <c r="B23" s="12" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>RPU_ON_SP237-HH150</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E23" s="9">
         <f t="shared" si="7"/>
@@ -3206,10 +3206,10 @@
         <v>1</v>
       </c>
       <c r="G23" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H23" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I23">
         <v>0</v>
@@ -3226,9 +3226,8 @@
       <c r="M23">
         <v>0</v>
       </c>
-      <c r="N23">
-        <f t="shared" si="8"/>
-        <v>2000000</v>
+      <c r="N23" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O23" s="10">
         <v>0</v>
@@ -3270,14 +3269,14 @@
     <row r="24" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A24" s="116"/>
       <c r="B24" s="12" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>RPU_ON_SP277-HH100</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E24" s="9">
         <f t="shared" si="7"/>
@@ -3287,10 +3286,10 @@
         <v>1</v>
       </c>
       <c r="G24" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H24" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I24">
         <v>0</v>
@@ -3307,9 +3306,8 @@
       <c r="M24">
         <v>0</v>
       </c>
-      <c r="N24">
-        <f t="shared" si="8"/>
-        <v>2000000</v>
+      <c r="N24" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O24" s="10">
         <v>0</v>
@@ -3351,14 +3349,14 @@
     <row r="25" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A25" s="116"/>
       <c r="B25" s="12" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>RPU_ON_SP277-HH150</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E25" s="9">
         <f t="shared" si="7"/>
@@ -3368,10 +3366,10 @@
         <v>1</v>
       </c>
       <c r="G25" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H25" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I25">
         <v>0</v>
@@ -3388,9 +3386,8 @@
       <c r="M25">
         <v>0</v>
       </c>
-      <c r="N25">
-        <f t="shared" si="8"/>
-        <v>2000000</v>
+      <c r="N25" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O25" s="10">
         <v>0</v>
@@ -3432,14 +3429,14 @@
     <row r="26" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A26" s="116"/>
       <c r="B26" s="12" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>RPU_ON_SP321-HH100</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E26" s="9">
         <f t="shared" si="7"/>
@@ -3449,10 +3446,10 @@
         <v>1</v>
       </c>
       <c r="G26" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H26" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I26">
         <v>0</v>
@@ -3469,9 +3466,8 @@
       <c r="M26">
         <v>0</v>
       </c>
-      <c r="N26">
-        <f t="shared" si="8"/>
-        <v>2000000</v>
+      <c r="N26" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O26" s="10">
         <v>0</v>
@@ -3513,14 +3509,14 @@
     <row r="27" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A27" s="116"/>
       <c r="B27" s="12" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>RPU_ON_SP321-HH150</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E27" s="9">
         <f t="shared" si="7"/>
@@ -3530,10 +3526,10 @@
         <v>1</v>
       </c>
       <c r="G27" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H27" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I27">
         <v>0</v>
@@ -3550,9 +3546,8 @@
       <c r="M27">
         <v>0</v>
       </c>
-      <c r="N27">
-        <f t="shared" si="8"/>
-        <v>2000000</v>
+      <c r="N27" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O27" s="10">
         <v>0</v>
@@ -3594,14 +3589,14 @@
     <row r="28" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A28" s="116"/>
       <c r="B28" s="12" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>RPU_OFF_SP379-HH100</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E28" s="9">
         <f t="shared" si="7"/>
@@ -3611,10 +3606,10 @@
         <v>1</v>
       </c>
       <c r="G28" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H28" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I28">
         <v>0</v>
@@ -3631,9 +3626,8 @@
       <c r="M28">
         <v>0</v>
       </c>
-      <c r="N28">
-        <f t="shared" si="8"/>
-        <v>2000000</v>
+      <c r="N28" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O28" s="10">
         <v>0</v>
@@ -3675,14 +3669,14 @@
     <row r="29" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A29" s="116"/>
       <c r="B29" s="12" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>RPU_OFF_SP379-HH150</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E29" s="9">
         <f t="shared" si="7"/>
@@ -3692,10 +3686,10 @@
         <v>1</v>
       </c>
       <c r="G29" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H29" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I29">
         <v>0</v>
@@ -3712,9 +3706,8 @@
       <c r="M29">
         <v>0</v>
       </c>
-      <c r="N29">
-        <f t="shared" si="8"/>
-        <v>2000000</v>
+      <c r="N29" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O29" s="10">
         <v>0</v>
@@ -3756,14 +3749,14 @@
     <row r="30" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A30" s="116"/>
       <c r="B30" s="12" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>RPU_OFF_SP450-HH100</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E30" s="9">
         <f t="shared" si="7"/>
@@ -3773,10 +3766,10 @@
         <v>1</v>
       </c>
       <c r="G30" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H30" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I30">
         <v>0</v>
@@ -3793,9 +3786,8 @@
       <c r="M30">
         <v>0</v>
       </c>
-      <c r="N30">
-        <f t="shared" si="8"/>
-        <v>2000000</v>
+      <c r="N30" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O30" s="10">
         <v>0</v>
@@ -3837,14 +3829,14 @@
     <row r="31" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A31" s="116"/>
       <c r="B31" s="12" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>RPU_OFF_SP450-HH150</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E31" s="9">
         <f t="shared" si="7"/>
@@ -3854,10 +3846,10 @@
         <v>1</v>
       </c>
       <c r="G31" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I31">
         <v>0</v>
@@ -3874,9 +3866,8 @@
       <c r="M31">
         <v>0</v>
       </c>
-      <c r="N31">
-        <f t="shared" si="8"/>
-        <v>2000000</v>
+      <c r="N31" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O31" s="10">
         <v>0</v>
@@ -3934,10 +3925,10 @@
         <v>1</v>
       </c>
       <c r="G32" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I32">
         <v>0</v>
@@ -3954,9 +3945,8 @@
       <c r="M32">
         <v>0</v>
       </c>
-      <c r="N32">
-        <f t="shared" si="8"/>
-        <v>2000000</v>
+      <c r="N32" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O32" s="10">
         <v>0</v>
@@ -3998,13 +3988,13 @@
     <row r="33" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A33" s="116"/>
       <c r="B33" s="12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C33" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="D33" s="7" t="s">
         <v>115</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>116</v>
       </c>
       <c r="E33" s="9">
         <f t="shared" si="7"/>
@@ -4014,10 +4004,10 @@
         <v>1</v>
       </c>
       <c r="G33" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H33" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I33">
         <v>0</v>
@@ -4034,8 +4024,8 @@
       <c r="M33">
         <v>0</v>
       </c>
-      <c r="N33">
-        <v>24000</v>
+      <c r="N33" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O33">
         <v>0</v>
@@ -4080,7 +4070,7 @@
         <v>13</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>26</v>
@@ -4093,10 +4083,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H34" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I34">
         <v>0</v>
@@ -4113,9 +4103,8 @@
       <c r="M34">
         <v>0</v>
       </c>
-      <c r="N34">
-        <f>N36/2</f>
-        <v>10000000</v>
+      <c r="N34" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O34" s="10">
         <v>0</v>
@@ -4160,7 +4149,7 @@
         <v>14</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>27</v>
@@ -4173,10 +4162,10 @@
         <v>1</v>
       </c>
       <c r="G35" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H35" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="H35" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="I35">
         <v>0</v>
@@ -4193,9 +4182,8 @@
       <c r="M35">
         <v>0</v>
       </c>
-      <c r="N35">
-        <f>3*N36</f>
-        <v>60000000</v>
+      <c r="N35" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O35" s="10">
         <v>0</v>
@@ -4240,7 +4228,7 @@
         <v>15</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>28</v>
@@ -4253,10 +4241,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I36">
         <v>0</v>
@@ -4273,8 +4261,8 @@
       <c r="M36">
         <v>0</v>
       </c>
-      <c r="N36">
-        <v>20000000</v>
+      <c r="N36" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="O36" s="10">
         <v>0</v>
@@ -4342,18 +4330,18 @@
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="14"/>
       <c r="B1" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B2" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C2" s="28">
         <v>18.600000000000001</v>
@@ -4365,30 +4353,30 @@
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="14"/>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" ref="C5:D5" si="0">C1&amp;"_"&amp;C3&amp;"_"&amp;C4</f>
@@ -4949,44 +4937,44 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="16" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="32" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D4" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E4" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="H4" s="16" t="s">
         <v>52</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="16" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="35"/>
       <c r="B5" s="16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>25</v>
@@ -4996,13 +4984,13 @@
         <v>Used (1 or 0)</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F5" s="16">
         <v>1</v>
       </c>
       <c r="G5" s="36" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H5" s="16">
         <f>INDEX(Data_base_case!$D$5:$Z$82,MATCH(Scenarios_definition!C5,Data_base_case!$D$5:$D$82,0),MATCH(Scenarios_definition!D5&amp;Scenarios_definition!G5,Data_base_case!$D$4:$Z$4,0))</f>
@@ -5015,17 +5003,17 @@
         <v>Semi-islanded</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C6" s="38" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D6" s="38" t="str">
         <f>Data_base_case!$Q$1</f>
         <v>Load min (% of max capacity)</v>
       </c>
       <c r="E6" s="38" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F6" s="38">
         <v>0</v>
@@ -5041,7 +5029,7 @@
     <row r="7" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="21"/>
       <c r="B7" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C7" s="1" t="str">
         <f>Data_base_case!D32</f>
@@ -5052,13 +5040,13 @@
         <v>Used (1 or 0)</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F7" s="1">
         <v>0</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H7" s="1">
         <f>INDEX(Data_base_case!$D$5:$Z$82,MATCH(Scenarios_definition!C7,Data_base_case!$D$5:$D$82,0),MATCH(Scenarios_definition!D7&amp;Scenarios_definition!G7,Data_base_case!$D$4:$Z$4,0))</f>
@@ -5067,20 +5055,20 @@
     </row>
     <row r="8" spans="1:8" s="30" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="21" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C8" s="30" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D8" s="30" t="str">
         <f>Data_base_case!$Q$1</f>
         <v>Load min (% of max capacity)</v>
       </c>
       <c r="E8" s="30" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F8" s="30">
         <v>1</v>
@@ -5096,17 +5084,17 @@
     <row r="9" spans="1:8" s="23" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="22"/>
       <c r="B9" s="23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D9" s="23" t="str">
         <f>Data_base_case!$Q$1</f>
         <v>Load min (% of max capacity)</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F9" s="23">
         <v>1</v>
@@ -5121,20 +5109,20 @@
     </row>
     <row r="10" spans="1:8" s="40" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B10" s="40" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D10" s="40" t="str">
         <f>Data_base_case!$Q$1</f>
         <v>Load min (% of max capacity)</v>
       </c>
       <c r="E10" s="40" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F10" s="40">
         <v>0</v>
@@ -5181,7 +5169,7 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B1" s="119" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C1" s="119"/>
       <c r="D1" s="119"/>
@@ -5195,47 +5183,47 @@
     </row>
     <row r="2" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="121" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C2" s="122" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G2" s="2">
         <v>2020</v>
       </c>
       <c r="H2" s="121" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K2" s="50" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B3" s="121"/>
       <c r="C3" s="122"/>
       <c r="D3" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="121"/>
       <c r="I3" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="50"/>
@@ -5244,7 +5232,7 @@
       <c r="B4" s="121"/>
       <c r="C4" s="122"/>
       <c r="D4" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E4" s="2"/>
       <c r="G4" s="2"/>
@@ -5269,7 +5257,7 @@
       <c r="O5" s="3"/>
       <c r="P5" s="29"/>
       <c r="Q5" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.35">
@@ -5283,61 +5271,61 @@
     </row>
     <row r="7" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="25" t="s">
-        <v>88</v>
-      </c>
-      <c r="C7" s="25" t="s">
-        <v>87</v>
-      </c>
-      <c r="D7" s="25" t="s">
-        <v>108</v>
-      </c>
-      <c r="E7" s="25" t="s">
+      <c r="F7" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="G7" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="H7" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="I7" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="F7" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="G7" s="25" t="s">
-        <v>95</v>
-      </c>
-      <c r="H7" s="25" t="s">
+      <c r="J7" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="K7" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="I7" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="J7" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="K7" s="26" t="s">
+      <c r="L7" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="L7" s="25" t="s">
+      <c r="M7" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="M7" s="25" t="s">
+      <c r="N7" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="N7" s="25" t="s">
+      <c r="O7" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="P7" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q7" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="O7" s="25" t="s">
-        <v>71</v>
-      </c>
-      <c r="P7" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q7" s="25" t="s">
-        <v>65</v>
-      </c>
       <c r="R7" s="25" t="s">
+        <v>151</v>
+      </c>
+      <c r="S7" s="25" t="s">
         <v>152</v>
-      </c>
-      <c r="S7" s="25" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.35">
@@ -5346,19 +5334,19 @@
         <v>1</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G8" s="49">
         <v>2020</v>
@@ -5368,13 +5356,13 @@
         <v>2019</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K8" s="17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L8" t="b">
         <v>0</v>
@@ -5407,19 +5395,19 @@
         <v>2</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G9" s="49">
         <v>2020</v>
@@ -5429,13 +5417,13 @@
         <v>2019</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K9" s="17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L9" t="b">
         <v>0</v>
@@ -5468,19 +5456,19 @@
         <v>3</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G10" s="49">
         <v>2020</v>
@@ -5490,13 +5478,13 @@
         <v>2019</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K10" s="17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L10" t="b">
         <v>0</v>
@@ -5529,19 +5517,19 @@
         <v>4</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G11" s="49">
         <v>2020</v>
@@ -5551,13 +5539,13 @@
         <v>2019</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K11" s="17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L11" t="b">
         <v>0</v>
@@ -5590,19 +5578,19 @@
         <v>5</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G12" s="49">
         <v>2020</v>
@@ -5612,13 +5600,13 @@
         <v>2019</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K12" s="17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L12" t="b">
         <v>0</v>
@@ -5651,19 +5639,19 @@
         <v>6</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G13" s="49">
         <v>2020</v>
@@ -5673,13 +5661,13 @@
         <v>2019</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K13" s="17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L13" t="b">
         <v>0</v>
@@ -5712,19 +5700,19 @@
         <v>7</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D14" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G14" s="49">
         <v>2020</v>
@@ -5734,13 +5722,13 @@
         <v>2019</v>
       </c>
       <c r="I14" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K14" s="17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L14" t="b">
         <v>0</v>
@@ -5773,19 +5761,19 @@
         <v>8</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G15" s="49">
         <v>2020</v>
@@ -5795,13 +5783,13 @@
         <v>2019</v>
       </c>
       <c r="I15" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K15" s="17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L15" t="b">
         <v>0</v>
@@ -5834,19 +5822,19 @@
         <v>9</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G16" s="49">
         <v>2020</v>
@@ -5856,13 +5844,13 @@
         <v>2019</v>
       </c>
       <c r="I16" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K16" s="17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L16" t="b">
         <v>0</v>
@@ -5895,19 +5883,19 @@
         <v>10</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G17" s="49">
         <v>2020</v>
@@ -5917,13 +5905,13 @@
         <v>2019</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K17" s="17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L17" t="b">
         <v>0</v>
@@ -5956,19 +5944,19 @@
         <v>11</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D18" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G18" s="49">
         <v>2020</v>
@@ -5978,13 +5966,13 @@
         <v>2019</v>
       </c>
       <c r="I18" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K18" s="17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L18" t="b">
         <v>0</v>
@@ -6017,19 +6005,19 @@
         <v>12</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G19" s="49">
         <v>2020</v>
@@ -6039,13 +6027,13 @@
         <v>2019</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J19" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K19" s="17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L19" t="b">
         <v>0</v>
@@ -6078,19 +6066,19 @@
         <v>13</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D20" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G20" s="49">
         <v>2020</v>
@@ -6100,13 +6088,13 @@
         <v>2019</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K20" s="17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L20" t="b">
         <v>0</v>
@@ -6139,19 +6127,19 @@
         <v>14</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D21" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G21" s="49">
         <v>2020</v>
@@ -6161,13 +6149,13 @@
         <v>2019</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J21" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K21" s="17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L21" t="b">
         <v>0</v>
@@ -6200,19 +6188,19 @@
         <v>15</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G22" s="49">
         <v>2020</v>
@@ -6222,13 +6210,13 @@
         <v>2019</v>
       </c>
       <c r="I22" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J22" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K22" s="17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L22" t="b">
         <v>0</v>
@@ -6261,19 +6249,19 @@
         <v>16</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D23" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G23" s="49">
         <v>2020</v>
@@ -6283,13 +6271,13 @@
         <v>2019</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J23" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K23" s="17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L23" t="b">
         <v>0</v>
@@ -6322,19 +6310,19 @@
         <v>17</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D24" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G24" s="49">
         <v>2020</v>
@@ -6344,13 +6332,13 @@
         <v>2019</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J24" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K24" s="17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L24" t="b">
         <v>0</v>
@@ -6383,19 +6371,19 @@
         <v>18</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G25" s="49">
         <v>2020</v>
@@ -6405,13 +6393,13 @@
         <v>2019</v>
       </c>
       <c r="I25" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J25" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K25" s="17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L25" t="b">
         <v>0</v>
@@ -6456,4 +6444,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{e4b931d8-a288-4db6-acc7-364bc8042050}" enabled="1" method="Privileged" siteId="{5218c2a1-81cc-40ce-af99-7505143bc263}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>